<commit_message>
Add 2026 mentoring program / move Kristina Weber to Alumni on BBS NextGen page and recompile
</commit_message>
<xml_diff>
--- a/data/roster_nextgen.xlsx
+++ b/data/roster_nextgen.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/widmelu1/Documents/git/bbs-basel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70657D8-3BAB-7F44-8EE3-BE22B7F6042F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E394025F-DF7C-9942-816C-107C3A4739CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="780" windowWidth="41120" windowHeight="24180" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020 Roster" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="41">
   <si>
     <t>First</t>
   </si>
@@ -88,15 +88,6 @@
   </si>
   <si>
     <t>Idorsia Pharmaceuticals Ltd</t>
-  </si>
-  <si>
-    <t>Kristina</t>
-  </si>
-  <si>
-    <t>Weber</t>
-  </si>
-  <si>
-    <t>mailing list</t>
   </si>
   <si>
     <t>Ottavia</t>
@@ -474,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="101.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" style="1" customWidth="1"/>
@@ -600,9 +591,7 @@
       <c r="E7" s="2">
         <v>1</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -612,7 +601,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" s="2">
         <v>1</v>
@@ -621,13 +610,13 @@
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E9" s="2">
         <v>1</v>
@@ -636,13 +625,13 @@
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" s="2">
         <v>1</v>
@@ -651,13 +640,13 @@
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="E11" s="2">
         <v>1</v>
@@ -702,36 +691,21 @@
         <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="E14" s="2">
         <v>1</v>
       </c>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="2">
-        <v>1</v>
-      </c>
-      <c r="F15" s="1"/>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D17" s="3"/>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D18" s="3"/>
     </row>
     <row r="19" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D19" s="3"/>
-    </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Update BBS NextGen committee and recompile
</commit_message>
<xml_diff>
--- a/data/roster_nextgen.xlsx
+++ b/data/roster_nextgen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/widmelu1/Documents/git/bbs-basel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E394025F-DF7C-9942-816C-107C3A4739CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25786D69-187F-4045-B2A8-708C8218A44A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>First</t>
   </si>
@@ -75,12 +75,6 @@
     <t>Papachristofi</t>
   </si>
   <si>
-    <t>Youyou</t>
-  </si>
-  <si>
-    <t>Hu</t>
-  </si>
-  <si>
     <t>Joana</t>
   </si>
   <si>
@@ -124,15 +118,6 @@
   </si>
   <si>
     <t>Celonic AG</t>
-  </si>
-  <si>
-    <t>Michal</t>
-  </si>
-  <si>
-    <t>Bechny</t>
-  </si>
-  <si>
-    <t>ETH Zürich</t>
   </si>
   <si>
     <t xml:space="preserve">Ainesh </t>
@@ -465,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="101.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" style="1" customWidth="1"/>
@@ -556,7 +541,7 @@
         <v>17</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E5" s="2">
         <v>1</v>
@@ -565,13 +550,13 @@
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2">
         <v>1</v>
@@ -580,13 +565,13 @@
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2">
         <v>1</v>
@@ -601,7 +586,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2">
         <v>1</v>
@@ -616,7 +601,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="E9" s="2">
         <v>1</v>
@@ -631,7 +616,7 @@
         <v>29</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E10" s="2">
         <v>1</v>
@@ -640,13 +625,13 @@
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" s="2">
         <v>1</v>
@@ -655,57 +640,27 @@
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2">
         <v>1</v>
       </c>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1</v>
-      </c>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="2">
-        <v>1</v>
-      </c>
-      <c r="F14" s="1"/>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D16" s="3"/>
     </row>
     <row r="17" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D17" s="3"/>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D18" s="3"/>
-    </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D19" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>